<commit_message>
Added Thermal pads for heatsinks in BOM.
Updated fab files
</commit_message>
<xml_diff>
--- a/Robot WallA/_output/Robot WallA.xlsx
+++ b/Robot WallA/_output/Robot WallA.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gdurand\_KiCad\Robot WallA\Robot WallA\_output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B35FABC6-2E78-41CF-931C-F51DC92CFEAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{689BBA7E-EDFC-4714-A941-9F65760549B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Robot WallA" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="304">
   <si>
     <t>Reference</t>
   </si>
@@ -346,9 +346,6 @@
     <t>SamacSys_Parts:64710ABEP</t>
   </si>
   <si>
-    <t>HS1,HS2</t>
-  </si>
-  <si>
     <t>374524B60023G</t>
   </si>
   <si>
@@ -920,12 +917,27 @@
   </si>
   <si>
     <t>Crystal:Crystal_SMD_3225-4Pin_3.2x2.5mm</t>
+  </si>
+  <si>
+    <t>H8,H9</t>
+  </si>
+  <si>
+    <t>ThermalPad</t>
+  </si>
+  <si>
+    <t>H6</t>
+  </si>
+  <si>
+    <t>H7</t>
+  </si>
+  <si>
+    <t>SPA2000-0.015-AC-62</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1464,15 +1476,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tableau1" displayName="Tableau1" ref="A1:F93" totalsRowShown="0">
-  <autoFilter ref="A1:F93"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tableau1" displayName="Tableau1" ref="A1:F95" totalsRowShown="0">
+  <autoFilter ref="A1:F95" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" name="Reference"/>
-    <tableColumn id="2" name="Qty"/>
-    <tableColumn id="3" name="Value"/>
-    <tableColumn id="4" name="Manufacturer_Part_Number"/>
-    <tableColumn id="5" name="Exclude from Board"/>
-    <tableColumn id="6" name="Footprint"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Reference"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Qty"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Value"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Manufacturer_Part_Number"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Exclude from Board"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Footprint"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1774,19 +1786,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F93"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F95"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="45.7109375" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="45.6640625" customWidth="1"/>
+    <col min="2" max="2" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="76.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1806,7 +1818,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1823,7 +1835,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1840,7 +1852,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1857,7 +1869,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1874,7 +1886,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1891,7 +1903,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -1908,7 +1920,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -1925,7 +1937,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -1942,7 +1954,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -1959,7 +1971,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>36</v>
       </c>
@@ -1976,7 +1988,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -1993,7 +2005,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>41</v>
       </c>
@@ -2010,7 +2022,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>44</v>
       </c>
@@ -2027,7 +2039,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>47</v>
       </c>
@@ -2044,7 +2056,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>50</v>
       </c>
@@ -2061,7 +2073,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>53</v>
       </c>
@@ -2078,7 +2090,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>57</v>
       </c>
@@ -2095,7 +2107,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>60</v>
       </c>
@@ -2112,7 +2124,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>64</v>
       </c>
@@ -2129,7 +2141,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>66</v>
       </c>
@@ -2146,7 +2158,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>70</v>
       </c>
@@ -2163,7 +2175,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>73</v>
       </c>
@@ -2180,7 +2192,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>76</v>
       </c>
@@ -2197,7 +2209,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>79</v>
       </c>
@@ -2214,7 +2226,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>82</v>
       </c>
@@ -2231,7 +2243,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>86</v>
       </c>
@@ -2248,7 +2260,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>89</v>
       </c>
@@ -2265,7 +2277,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>92</v>
       </c>
@@ -2282,7 +2294,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>96</v>
       </c>
@@ -2299,7 +2311,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>99</v>
       </c>
@@ -2316,7 +2328,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>103</v>
       </c>
@@ -2333,7 +2345,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>105</v>
       </c>
@@ -2350,1024 +2362,1058 @@
         <v>107</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>301</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>300</v>
+      </c>
+      <c r="D34" t="s">
+        <v>303</v>
+      </c>
+      <c r="E34" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>302</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>300</v>
+      </c>
+      <c r="D35">
+        <v>404035125</v>
+      </c>
+      <c r="E35" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>299</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
         <v>108</v>
       </c>
-      <c r="B34">
+      <c r="D36" t="s">
+        <v>108</v>
+      </c>
+      <c r="F36" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>110</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>111</v>
+      </c>
+      <c r="D37" t="s">
+        <v>111</v>
+      </c>
+      <c r="F37" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>113</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>114</v>
+      </c>
+      <c r="D38" t="s">
+        <v>114</v>
+      </c>
+      <c r="F38" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>116</v>
+      </c>
+      <c r="B39">
         <v>2</v>
       </c>
-      <c r="C34" t="s">
-        <v>109</v>
-      </c>
-      <c r="D34" t="s">
-        <v>109</v>
-      </c>
-      <c r="F34" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>111</v>
-      </c>
-      <c r="B35">
-        <v>1</v>
-      </c>
-      <c r="C35" t="s">
-        <v>112</v>
-      </c>
-      <c r="D35" t="s">
-        <v>112</v>
-      </c>
-      <c r="F35" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>114</v>
-      </c>
-      <c r="B36">
-        <v>1</v>
-      </c>
-      <c r="C36" t="s">
-        <v>115</v>
-      </c>
-      <c r="D36" t="s">
-        <v>115</v>
-      </c>
-      <c r="F36" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+      <c r="C39" t="s">
         <v>117</v>
       </c>
-      <c r="B37">
-        <v>2</v>
-      </c>
-      <c r="C37" t="s">
+      <c r="D39" t="s">
+        <v>117</v>
+      </c>
+      <c r="F39" t="s">
         <v>118</v>
       </c>
-      <c r="D37" t="s">
-        <v>118</v>
-      </c>
-      <c r="F37" t="s">
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
         <v>120</v>
       </c>
-      <c r="B38">
-        <v>1</v>
-      </c>
-      <c r="C38" t="s">
+      <c r="D40" t="s">
+        <v>120</v>
+      </c>
+      <c r="F40" t="s">
         <v>121</v>
       </c>
-      <c r="D38" t="s">
-        <v>121</v>
-      </c>
-      <c r="F38" t="s">
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
         <v>123</v>
       </c>
-      <c r="B39">
-        <v>1</v>
-      </c>
-      <c r="C39" t="s">
+      <c r="D41" t="s">
+        <v>123</v>
+      </c>
+      <c r="F41" t="s">
         <v>124</v>
       </c>
-      <c r="D39" t="s">
-        <v>124</v>
-      </c>
-      <c r="F39" t="s">
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+      <c r="B42">
+        <v>1</v>
+      </c>
+      <c r="C42" t="s">
         <v>126</v>
       </c>
-      <c r="B40">
-        <v>1</v>
-      </c>
-      <c r="C40" t="s">
+      <c r="D42" t="s">
+        <v>126</v>
+      </c>
+      <c r="F42" t="s">
         <v>127</v>
       </c>
-      <c r="D40" t="s">
-        <v>127</v>
-      </c>
-      <c r="F40" t="s">
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+      <c r="B43">
+        <v>1</v>
+      </c>
+      <c r="C43" t="s">
         <v>129</v>
       </c>
-      <c r="B41">
-        <v>1</v>
-      </c>
-      <c r="C41" t="s">
+      <c r="D43" t="s">
+        <v>129</v>
+      </c>
+      <c r="F43" t="s">
         <v>130</v>
       </c>
-      <c r="D41" t="s">
-        <v>130</v>
-      </c>
-      <c r="F41" t="s">
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
         <v>131</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>132</v>
-      </c>
-      <c r="B42">
-        <v>4</v>
-      </c>
-      <c r="C42" t="s">
-        <v>133</v>
-      </c>
-      <c r="D42" t="s">
-        <v>133</v>
-      </c>
-      <c r="F42" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>135</v>
-      </c>
-      <c r="B43">
-        <v>2</v>
-      </c>
-      <c r="C43" t="s">
-        <v>136</v>
-      </c>
-      <c r="D43" t="s">
-        <v>136</v>
-      </c>
-      <c r="F43" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>138</v>
       </c>
       <c r="B44">
         <v>4</v>
       </c>
       <c r="C44" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D44" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F44" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="B45">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C45" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="D45" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="F45" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="B46">
         <v>4</v>
       </c>
       <c r="C46" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="D46" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="F46" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="B47">
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="D47" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="F47" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="B48">
         <v>4</v>
       </c>
       <c r="C48" t="s">
+        <v>144</v>
+      </c>
+      <c r="D48" t="s">
+        <v>144</v>
+      </c>
+      <c r="F48" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>146</v>
+      </c>
+      <c r="B49">
+        <v>1</v>
+      </c>
+      <c r="C49" t="s">
+        <v>147</v>
+      </c>
+      <c r="D49" t="s">
+        <v>147</v>
+      </c>
+      <c r="F49" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>149</v>
+      </c>
+      <c r="B50">
+        <v>4</v>
+      </c>
+      <c r="C50" t="s">
+        <v>150</v>
+      </c>
+      <c r="D50" t="s">
+        <v>150</v>
+      </c>
+      <c r="F50" t="s">
         <v>151</v>
       </c>
-      <c r="D48" t="s">
-        <v>151</v>
-      </c>
-      <c r="F48" t="s">
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
         <v>152</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>153</v>
-      </c>
-      <c r="B49">
-        <v>4</v>
-      </c>
-      <c r="C49" t="s">
-        <v>154</v>
-      </c>
-      <c r="D49" t="s">
-        <v>155</v>
-      </c>
-      <c r="F49" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>157</v>
-      </c>
-      <c r="B50">
-        <v>1</v>
-      </c>
-      <c r="C50" t="s">
-        <v>158</v>
-      </c>
-      <c r="D50" t="s">
-        <v>159</v>
-      </c>
-      <c r="F50" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>161</v>
       </c>
       <c r="B51">
         <v>4</v>
       </c>
       <c r="C51" t="s">
+        <v>153</v>
+      </c>
+      <c r="D51" t="s">
+        <v>154</v>
+      </c>
+      <c r="F51" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>156</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
+        <v>157</v>
+      </c>
+      <c r="D52" t="s">
+        <v>158</v>
+      </c>
+      <c r="F52" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>160</v>
+      </c>
+      <c r="B53">
+        <v>4</v>
+      </c>
+      <c r="C53" t="s">
+        <v>161</v>
+      </c>
+      <c r="D53" t="s">
         <v>162</v>
       </c>
-      <c r="D51" t="s">
+      <c r="F53" t="s">
         <v>163</v>
       </c>
-      <c r="F51" t="s">
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
         <v>164</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>165</v>
-      </c>
-      <c r="B52">
-        <v>2</v>
-      </c>
-      <c r="C52" t="s">
-        <v>166</v>
-      </c>
-      <c r="D52" t="s">
-        <v>166</v>
-      </c>
-      <c r="F52" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>168</v>
-      </c>
-      <c r="B53">
-        <v>1</v>
-      </c>
-      <c r="C53" t="s">
-        <v>169</v>
-      </c>
-      <c r="D53" t="s">
-        <v>170</v>
-      </c>
-      <c r="F53" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>172</v>
       </c>
       <c r="B54">
         <v>2</v>
       </c>
       <c r="C54" t="s">
+        <v>165</v>
+      </c>
+      <c r="D54" t="s">
+        <v>165</v>
+      </c>
+      <c r="F54" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>167</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="C55" t="s">
+        <v>168</v>
+      </c>
+      <c r="D55" t="s">
+        <v>169</v>
+      </c>
+      <c r="F55" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>171</v>
+      </c>
+      <c r="B56">
+        <v>2</v>
+      </c>
+      <c r="C56" t="s">
+        <v>172</v>
+      </c>
+      <c r="D56" t="s">
         <v>173</v>
       </c>
-      <c r="D54" t="s">
+      <c r="F56" t="s">
         <v>174</v>
       </c>
-      <c r="F54" t="s">
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+      <c r="B57">
+        <v>11</v>
+      </c>
+      <c r="C57" t="s">
         <v>176</v>
       </c>
-      <c r="B55">
-        <v>11</v>
-      </c>
-      <c r="C55" t="s">
+      <c r="D57" t="s">
         <v>177</v>
       </c>
-      <c r="D55" t="s">
+      <c r="E57" t="s">
         <v>178</v>
       </c>
-      <c r="E55" t="s">
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
         <v>179</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>180</v>
-      </c>
-      <c r="B56">
-        <v>4</v>
-      </c>
-      <c r="C56" t="s">
-        <v>181</v>
-      </c>
-      <c r="D56" t="s">
-        <v>182</v>
-      </c>
-      <c r="E56" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>183</v>
-      </c>
-      <c r="B57">
-        <v>2</v>
-      </c>
-      <c r="C57" t="s">
-        <v>181</v>
-      </c>
-      <c r="D57" t="s">
-        <v>184</v>
-      </c>
-      <c r="E57" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>185</v>
       </c>
       <c r="B58">
         <v>4</v>
       </c>
       <c r="C58" t="s">
+        <v>180</v>
+      </c>
+      <c r="D58" t="s">
+        <v>181</v>
+      </c>
+      <c r="E58" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>182</v>
+      </c>
+      <c r="B59">
+        <v>2</v>
+      </c>
+      <c r="C59" t="s">
+        <v>180</v>
+      </c>
+      <c r="D59" t="s">
+        <v>183</v>
+      </c>
+      <c r="E59" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>184</v>
+      </c>
+      <c r="B60">
+        <v>4</v>
+      </c>
+      <c r="C60" t="s">
+        <v>185</v>
+      </c>
+      <c r="D60" t="s">
+        <v>185</v>
+      </c>
+      <c r="F60" t="s">
         <v>186</v>
       </c>
-      <c r="D58" t="s">
-        <v>186</v>
-      </c>
-      <c r="F58" t="s">
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+      <c r="B61">
+        <v>4</v>
+      </c>
+      <c r="C61" t="s">
         <v>188</v>
       </c>
-      <c r="B59">
-        <v>4</v>
-      </c>
-      <c r="C59" t="s">
+      <c r="D61" t="s">
         <v>189</v>
-      </c>
-      <c r="D59" t="s">
-        <v>190</v>
-      </c>
-      <c r="F59" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>191</v>
-      </c>
-      <c r="B60">
-        <v>2</v>
-      </c>
-      <c r="C60" t="s">
-        <v>192</v>
-      </c>
-      <c r="D60" t="s">
-        <v>193</v>
-      </c>
-      <c r="F60" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>194</v>
-      </c>
-      <c r="B61">
-        <v>1</v>
-      </c>
-      <c r="C61" t="s">
-        <v>195</v>
-      </c>
-      <c r="D61" t="s">
-        <v>196</v>
       </c>
       <c r="F61" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="B62">
         <v>2</v>
       </c>
       <c r="C62" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="D62" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="F62" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="B63">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C63" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="D63" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="F63" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="B64">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C64" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="D64" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="F64" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="B65">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C65" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="D65" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="F65" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="B66">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C66" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="D66" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="F66" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="B67">
         <v>1</v>
       </c>
       <c r="C67" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="D67" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="F67" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="B68">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C68" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="D68" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="F68" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="B69">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C69" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="D69" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="F69" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="B70">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C70" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="D70" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="F70" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="B71">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C71" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="D71" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="F71" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B72">
         <v>1</v>
       </c>
       <c r="C72" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="D72" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="F72" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B73">
         <v>1</v>
       </c>
       <c r="C73" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="D73" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="F73" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="B74">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C74" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="D74" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="F74" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="B75">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C75" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="D75" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="F75" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="B76">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C76" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="D76" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="F76" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="B77">
         <v>2</v>
       </c>
       <c r="C77" t="s">
-        <v>210</v>
+        <v>237</v>
       </c>
       <c r="D77" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="F77" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="B78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C78" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="D78" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="F78" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="B79">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C79" t="s">
-        <v>249</v>
+        <v>209</v>
       </c>
       <c r="D79" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="F79" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="B80">
         <v>1</v>
       </c>
       <c r="C80" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="D80" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="F80" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="B81">
         <v>1</v>
       </c>
       <c r="C81" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="D81" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="F81" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="B82">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C82" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="D82" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="F82" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
+        <v>253</v>
+      </c>
+      <c r="B83">
+        <v>1</v>
+      </c>
+      <c r="C83" t="s">
+        <v>254</v>
+      </c>
+      <c r="D83" t="s">
+        <v>255</v>
+      </c>
+      <c r="F83" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>256</v>
+      </c>
+      <c r="B84">
+        <v>12</v>
+      </c>
+      <c r="C84" t="s">
+        <v>257</v>
+      </c>
+      <c r="D84" t="s">
+        <v>258</v>
+      </c>
+      <c r="F84" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>259</v>
+      </c>
+      <c r="B85">
+        <v>1</v>
+      </c>
+      <c r="C85" t="s">
         <v>260</v>
       </c>
-      <c r="B83">
-        <v>1</v>
-      </c>
-      <c r="C83" t="s">
+      <c r="D85" t="s">
         <v>261</v>
       </c>
-      <c r="D83" t="s">
+      <c r="F85" t="s">
         <v>262</v>
       </c>
-      <c r="F83" t="s">
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
+      <c r="B86">
+        <v>1</v>
+      </c>
+      <c r="C86" t="s">
         <v>264</v>
       </c>
-      <c r="B84">
-        <v>1</v>
-      </c>
-      <c r="C84" t="s">
+      <c r="D86" t="s">
         <v>265</v>
       </c>
-      <c r="D84" t="s">
+      <c r="F86" t="s">
         <v>266</v>
       </c>
-      <c r="F84" t="s">
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
+      <c r="B87">
+        <v>1</v>
+      </c>
+      <c r="C87" t="s">
         <v>268</v>
       </c>
-      <c r="B85">
-        <v>1</v>
-      </c>
-      <c r="C85" t="s">
+      <c r="D87" t="s">
+        <v>268</v>
+      </c>
+      <c r="F87" t="s">
         <v>269</v>
       </c>
-      <c r="D85" t="s">
-        <v>269</v>
-      </c>
-      <c r="F85" t="s">
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
         <v>271</v>
       </c>
-      <c r="B86">
-        <v>3</v>
-      </c>
-      <c r="C86" t="s">
+      <c r="D88" t="s">
         <v>272</v>
       </c>
-      <c r="D86" t="s">
+      <c r="F88" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
         <v>273</v>
       </c>
-      <c r="F86" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
+      <c r="B89">
+        <v>1</v>
+      </c>
+      <c r="C89" t="s">
         <v>274</v>
       </c>
-      <c r="B87">
-        <v>1</v>
-      </c>
-      <c r="C87" t="s">
+      <c r="D89" t="s">
         <v>275</v>
       </c>
-      <c r="D87" t="s">
+      <c r="F89" t="s">
         <v>276</v>
       </c>
-      <c r="F87" t="s">
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
+      <c r="B90">
+        <v>4</v>
+      </c>
+      <c r="C90" t="s">
         <v>278</v>
       </c>
-      <c r="B88">
-        <v>4</v>
-      </c>
-      <c r="C88" t="s">
+      <c r="D90" t="s">
+        <v>278</v>
+      </c>
+      <c r="F90" t="s">
         <v>279</v>
       </c>
-      <c r="D88" t="s">
-        <v>279</v>
-      </c>
-      <c r="F88" t="s">
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
+      <c r="B91">
+        <v>1</v>
+      </c>
+      <c r="C91" t="s">
         <v>281</v>
       </c>
-      <c r="B89">
-        <v>1</v>
-      </c>
-      <c r="C89" t="s">
+      <c r="D91" t="s">
+        <v>281</v>
+      </c>
+      <c r="F91" t="s">
         <v>282</v>
       </c>
-      <c r="D89" t="s">
-        <v>282</v>
-      </c>
-      <c r="F89" t="s">
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
+      <c r="B92">
+        <v>1</v>
+      </c>
+      <c r="C92" t="s">
         <v>284</v>
       </c>
-      <c r="B90">
-        <v>1</v>
-      </c>
-      <c r="C90" t="s">
+      <c r="D92" t="s">
         <v>285</v>
       </c>
-      <c r="D90" t="s">
+      <c r="F92" t="s">
         <v>286</v>
       </c>
-      <c r="F90" t="s">
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
         <v>288</v>
       </c>
-      <c r="B91">
-        <v>1</v>
-      </c>
-      <c r="C91" t="s">
+      <c r="D93" t="s">
         <v>289</v>
       </c>
-      <c r="D91" t="s">
+      <c r="F93" t="s">
         <v>290</v>
       </c>
-      <c r="F91" t="s">
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
+      <c r="B94">
+        <v>2</v>
+      </c>
+      <c r="C94" t="s">
         <v>292</v>
       </c>
-      <c r="B92">
-        <v>2</v>
-      </c>
-      <c r="C92" t="s">
+      <c r="D94" t="s">
         <v>293</v>
       </c>
-      <c r="D92" t="s">
+      <c r="F94" t="s">
         <v>294</v>
       </c>
-      <c r="F92" t="s">
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
+      <c r="B95">
+        <v>1</v>
+      </c>
+      <c r="C95" t="s">
         <v>296</v>
       </c>
-      <c r="B93">
-        <v>1</v>
-      </c>
-      <c r="C93" t="s">
+      <c r="D95" t="s">
         <v>297</v>
       </c>
-      <c r="D93" t="s">
+      <c r="F95" t="s">
         <v>298</v>
-      </c>
-      <c r="F93" t="s">
-        <v>299</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrected schematic labels encoders according to PCB labels... (inversion...)
Add fab files
cleaned
</commit_message>
<xml_diff>
--- a/Robot WallA/_output/Robot WallA.xlsx
+++ b/Robot WallA/_output/Robot WallA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gdurand\_KiCad\Robot WallA\Robot WallA\_output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD4ABF34-4C0D-49FE-8B78-576A73E9B000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C89E976D-4B1A-480B-B733-C27050AB0572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Robot WallA" sheetId="1" r:id="rId1"/>
@@ -1469,11 +1469,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20 % - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1549,9 +1548,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1589,7 +1588,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1695,7 +1694,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1837,7 +1836,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3606,11 +3605,8 @@
         <v>316</v>
       </c>
     </row>
-    <row r="115" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C115" s="2"/>
-    </row>
     <row r="116" spans="3:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C116" s="3"/>
+      <c r="C116" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>